<commit_message>
Prvi zvanicni testovi, promena imena racuna
</commit_message>
<xml_diff>
--- a/testdata/execute.xlsx
+++ b/testdata/execute.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="30">
   <si>
     <t>App</t>
   </si>
@@ -110,10 +110,16 @@
     <t>C70826</t>
   </si>
   <si>
-    <t>Change_Name_Of_Account_RSD[MOB_ANDROID]</t>
+    <t>Accounts-Domestic_Accounts-Change_name_of_account_[MOB]</t>
   </si>
   <si>
     <t>C70827</t>
+  </si>
+  <si>
+    <t>Accounts-Domestic_Accounts-Change_name_of_account_to_default_[MOB]</t>
+  </si>
+  <si>
+    <t>C70828</t>
   </si>
 </sst>
 </file>
@@ -787,7 +793,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -798,6 +804,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1129,7 +1136,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="6"/>
   <cols>
     <col min="2" max="2" width="112.574074074074" customWidth="1"/>
@@ -1343,14 +1350,37 @@
         <v>13</v>
       </c>
     </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G8" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
-  <conditionalFormatting sqref="C2:C9">
+  <conditionalFormatting sqref="C2:C10">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1 C10:C1048576">
+  <conditionalFormatting sqref="C1 C11:C1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="7"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
brisanje nepotrebnih wait koraka
</commit_message>
<xml_diff>
--- a/testdata/execute.xlsx
+++ b/testdata/execute.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="33">
   <si>
     <t>App</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>Accounts-Foreign_Accounts-Change_name_of_account_to_default_[MOB]</t>
+  </si>
+  <si>
+    <t>Homepage_Bottom_nav_[MOB_ANDROID]</t>
   </si>
 </sst>
 </file>
@@ -1140,7 +1143,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="6"/>
   <cols>
     <col min="2" max="2" width="112.574074074074" customWidth="1"/>
@@ -1423,18 +1426,44 @@
         <v>13</v>
       </c>
     </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G10" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G12" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
+  <conditionalFormatting sqref="C13">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C2:C10">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11:C12">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C11:C12">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1 C13:C1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="8"/>
+  <conditionalFormatting sqref="C1 C14:C1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="9"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>